<commit_message>
Add BSCR settings and schedule staging tabs
</commit_message>
<xml_diff>
--- a/bscr/workbooks/Workings_with_geocodingFW - Including blanks USD.xlsx
+++ b/bscr/workbooks/Workings_with_geocodingFW - Including blanks USD.xlsx
@@ -1,43 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns6="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent>
-    <mc:Choice Requires="x15">
-      <x15ac:absPath url="W:\Cat Modelling\Group Reporting\Reports\2026\2026-01 - BSCR\UKEU\Workings\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30AD028F-592B-4888-AD91-FB2F3163888C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <ns1:AlternateContent>
+    <ns1:Choice Requires="x15">
+      <ns2:absPath url="W:\Cat Modelling\Group Reporting\Reports\2026\2026-01 - BSCR\UKEU\Workings\"/>
+    </ns1:Choice>
+  </ns1:AlternateContent>
+  <ns3:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30AD028F-592B-4888-AD91-FB2F3163888C}" ns4:coauthVersionLast="47" ns4:coauthVersionMax="47" ns5:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="3" xr2:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21240" activeTab="3" ns6:uid="{33ED103A-C225-4AF7-8380-A17D5970A431}"/>
   </bookViews>
   <sheets>
     <sheet name="piv" sheetId="2" r:id="rId1"/>
     <sheet name="output" sheetId="1" r:id="rId2"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
     <sheet name="AUDIT_SUMMARY" sheetId="4" r:id="rId10"/>
+    <sheet name="Settings" sheetId="5" r:id="rId11"/>
+    <sheet name="Schedule X(a)" sheetId="6" r:id="rId12"/>
+    <sheet name="Schedule X(b)" sheetId="7" r:id="rId13"/>
+    <sheet name="Schedule X(c)" sheetId="8" r:id="rId14"/>
+    <sheet name="Schedule X(f)" sheetId="9" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">output!$A$1:$F$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Sheet1!$A$1:$K$1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId4"/>
     <pivotCache cacheId="39" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+      <ns8:calcFeatures>
+        <ns8:feature name="microsoft.com:RD"/>
+        <ns8:feature name="microsoft.com:Single"/>
+        <ns8:feature name="microsoft.com:FV"/>
+        <ns8:feature name="microsoft.com:CNMTM"/>
+        <ns8:feature name="microsoft.com:LET_WF"/>
+        <ns8:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns8:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns8:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -1182,7 +1187,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Richard Hampton" refreshedDate="46090.700917708331" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="49" xr:uid="{B1A2DC09-0005-4103-9A04-052000D9B748}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" refreshOnLoad="1" mc:Ignorable="xr" r:id="rId1" refreshedBy="Richard Hampton" refreshedDate="46090.700917708331" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="49" xr:uid="{B1A2DC09-0005-4103-9A04-052000D9B748}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:J50" sheet="output"/>
   </cacheSource>
@@ -1290,7 +1295,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Faye Williams" refreshedDate="46106.622011574073" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="453" xr:uid="{8B38D0A1-59CD-453E-BBD5-7D49D4105093}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" refreshOnLoad="1" mc:Ignorable="xr" r:id="rId1" refreshedBy="Faye Williams" refreshedDate="46106.622011574073" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="453" xr:uid="{8B38D0A1-59CD-453E-BBD5-7D49D4105093}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:K1048576" sheet="Sheet1"/>
   </cacheSource>
@@ -10560,23 +10565,26 @@
         <v>6</v>
       </c>
       <c r="C2" s="1">
-        <v>4645929142.0892601</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A2,'Sheet1'!$C:$C,$B2,'Sheet1'!$G:$G,$F2)</f>
+        <v>4645929142.03575</v>
       </c>
       <c r="D2" s="1">
-        <v>2931952651.35181</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A2,'Sheet1'!$C:$C,$B2,'Sheet1'!$G:$G,$F2)</f>
+        <v>2931952651.02002</v>
       </c>
       <c r="E2">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A2,'Sheet1'!$C:$C,$B2,'Sheet1'!$G:$G,$F2)</f>
         <v>663</v>
       </c>
       <c r="F2">
         <v>0</v>
       </c>
       <c r="G2" s="7">
-        <f>C2*1.35</f>
+        <f>C2*Settings!$B$3</f>
         <v>6272004341.8205013</v>
       </c>
       <c r="H2" s="1">
-        <f>D2*1.35</f>
+        <f>D2*Settings!$B$3</f>
         <v>3958136079.3249435</v>
       </c>
       <c r="I2" s="7">
@@ -10596,12 +10604,15 @@
         <v>6</v>
       </c>
       <c r="C3" s="1">
-        <v>25152755367.618698</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A3,'Sheet1'!$C:$C,$B3,'Sheet1'!$G:$G,$F3)</f>
+        <v>25152755366.6675</v>
       </c>
       <c r="D3" s="1">
-        <v>18626528497.776199</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A3,'Sheet1'!$C:$C,$B3,'Sheet1'!$G:$G,$F3)</f>
+        <v>18626528497.3074</v>
       </c>
       <c r="E3">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A3,'Sheet1'!$C:$C,$B3,'Sheet1'!$G:$G,$F3)</f>
         <v>4678</v>
       </c>
       <c r="F3">
@@ -10632,12 +10643,15 @@
         <v>6</v>
       </c>
       <c r="C4">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A4,'Sheet1'!$C:$C,$B4,'Sheet1'!$G:$G,$F4)</f>
         <v>1652000</v>
       </c>
       <c r="D4">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A4,'Sheet1'!$C:$C,$B4,'Sheet1'!$G:$G,$F4)</f>
         <v>1652000</v>
       </c>
       <c r="E4">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A4,'Sheet1'!$C:$C,$B4,'Sheet1'!$G:$G,$F4)</f>
         <v>9</v>
       </c>
       <c r="F4">
@@ -10668,12 +10682,15 @@
         <v>6</v>
       </c>
       <c r="C5">
-        <v>20414496.800000001</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A5,'Sheet1'!$C:$C,$B5,'Sheet1'!$G:$G,$F5)</f>
+        <v>20414496.8</v>
       </c>
       <c r="D5">
-        <v>20414496.800000001</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A5,'Sheet1'!$C:$C,$B5,'Sheet1'!$G:$G,$F5)</f>
+        <v>20414496.8</v>
       </c>
       <c r="E5">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A5,'Sheet1'!$C:$C,$B5,'Sheet1'!$G:$G,$F5)</f>
         <v>27</v>
       </c>
       <c r="F5">
@@ -10704,12 +10721,15 @@
         <v>6</v>
       </c>
       <c r="C6">
-        <v>15433806.3999999</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A6,'Sheet1'!$C:$C,$B6,'Sheet1'!$G:$G,$F6)</f>
+        <v>15433806.4</v>
       </c>
       <c r="D6">
-        <v>15433806.3999999</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A6,'Sheet1'!$C:$C,$B6,'Sheet1'!$G:$G,$F6)</f>
+        <v>15433806.4</v>
       </c>
       <c r="E6">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A6,'Sheet1'!$C:$C,$B6,'Sheet1'!$G:$G,$F6)</f>
         <v>29</v>
       </c>
       <c r="F6">
@@ -10740,12 +10760,15 @@
         <v>6</v>
       </c>
       <c r="C7">
-        <v>121727653503.479</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A7,'Sheet1'!$C:$C,$B7,'Sheet1'!$G:$G,$F7)</f>
+        <v>121728008563.88</v>
       </c>
       <c r="D7">
-        <v>121727653503.479</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A7,'Sheet1'!$C:$C,$B7,'Sheet1'!$G:$G,$F7)</f>
+        <v>121728008563.88</v>
       </c>
       <c r="E7">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A7,'Sheet1'!$C:$C,$B7,'Sheet1'!$G:$G,$F7)</f>
         <v>173658</v>
       </c>
       <c r="F7">
@@ -10776,12 +10799,15 @@
         <v>6</v>
       </c>
       <c r="C8">
-        <v>699027304.74033594</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A8,'Sheet1'!$C:$C,$B8,'Sheet1'!$G:$G,$F8)</f>
+        <v>699027304.76611</v>
       </c>
       <c r="D8">
-        <v>406962151.02545899</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A8,'Sheet1'!$C:$C,$B8,'Sheet1'!$G:$G,$F8)</f>
+        <v>406962151.02611</v>
       </c>
       <c r="E8">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A8,'Sheet1'!$C:$C,$B8,'Sheet1'!$G:$G,$F8)</f>
         <v>55</v>
       </c>
       <c r="F8">
@@ -10812,12 +10838,15 @@
         <v>6</v>
       </c>
       <c r="C9">
-        <v>7347517214.2083597</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A9,'Sheet1'!$C:$C,$B9,'Sheet1'!$G:$G,$F9)</f>
+        <v>7347517214.04485</v>
       </c>
       <c r="D9">
-        <v>5831772777.3838902</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A9,'Sheet1'!$C:$C,$B9,'Sheet1'!$G:$G,$F9)</f>
+        <v>5831772777.39485</v>
       </c>
       <c r="E9">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A9,'Sheet1'!$C:$C,$B9,'Sheet1'!$G:$G,$F9)</f>
         <v>1915</v>
       </c>
       <c r="F9">
@@ -10848,12 +10877,15 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <v>349291128.70019001</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A10,'Sheet1'!$C:$C,$B10,'Sheet1'!$G:$G,$F10)</f>
+        <v>349291128.7</v>
       </c>
       <c r="D10">
-        <v>349291128.70019001</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A10,'Sheet1'!$C:$C,$B10,'Sheet1'!$G:$G,$F10)</f>
+        <v>349291128.7</v>
       </c>
       <c r="E10">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A10,'Sheet1'!$C:$C,$B10,'Sheet1'!$G:$G,$F10)</f>
         <v>201</v>
       </c>
       <c r="F10">
@@ -10884,12 +10916,15 @@
         <v>6</v>
       </c>
       <c r="C11">
-        <v>77211907517.555206</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A11,'Sheet1'!$C:$C,$B11,'Sheet1'!$G:$G,$F11)</f>
+        <v>77211907518.142</v>
       </c>
       <c r="D11">
-        <v>75515308379.152496</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A11,'Sheet1'!$C:$C,$B11,'Sheet1'!$G:$G,$F11)</f>
+        <v>75515308381.742</v>
       </c>
       <c r="E11">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A11,'Sheet1'!$C:$C,$B11,'Sheet1'!$G:$G,$F11)</f>
         <v>89851</v>
       </c>
       <c r="F11">
@@ -10920,12 +10955,15 @@
         <v>10</v>
       </c>
       <c r="C12" s="1">
-        <v>591803570.79433501</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A12,'Sheet1'!$C:$C,$B12,'Sheet1'!$G:$G,$F12)</f>
+        <v>591803570.7403</v>
       </c>
       <c r="D12" s="1">
-        <v>395404009.10095602</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A12,'Sheet1'!$C:$C,$B12,'Sheet1'!$G:$G,$F12)</f>
+        <v>395404009.102</v>
       </c>
       <c r="E12">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A12,'Sheet1'!$C:$C,$B12,'Sheet1'!$G:$G,$F12)</f>
         <v>46</v>
       </c>
       <c r="F12">
@@ -10956,12 +10994,15 @@
         <v>10</v>
       </c>
       <c r="C13" s="1">
-        <v>15621176039.304501</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A13,'Sheet1'!$C:$C,$B13,'Sheet1'!$G:$G,$F13)</f>
+        <v>15621176039.34</v>
       </c>
       <c r="D13" s="1">
-        <v>12132651704.075899</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A13,'Sheet1'!$C:$C,$B13,'Sheet1'!$G:$G,$F13)</f>
+        <v>12132651704.25</v>
       </c>
       <c r="E13">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A13,'Sheet1'!$C:$C,$B13,'Sheet1'!$G:$G,$F13)</f>
         <v>2767</v>
       </c>
       <c r="F13">
@@ -10992,12 +11033,15 @@
         <v>10</v>
       </c>
       <c r="C14">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A14,'Sheet1'!$C:$C,$B14,'Sheet1'!$G:$G,$F14)</f>
         <v>5578000</v>
       </c>
       <c r="D14">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A14,'Sheet1'!$C:$C,$B14,'Sheet1'!$G:$G,$F14)</f>
         <v>5578000</v>
       </c>
       <c r="E14">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A14,'Sheet1'!$C:$C,$B14,'Sheet1'!$G:$G,$F14)</f>
         <v>5</v>
       </c>
       <c r="F14">
@@ -11028,12 +11072,15 @@
         <v>10</v>
       </c>
       <c r="C15">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A15,'Sheet1'!$C:$C,$B15,'Sheet1'!$G:$G,$F15)</f>
         <v>7099946</v>
       </c>
       <c r="D15">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A15,'Sheet1'!$C:$C,$B15,'Sheet1'!$G:$G,$F15)</f>
         <v>7099946</v>
       </c>
       <c r="E15">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A15,'Sheet1'!$C:$C,$B15,'Sheet1'!$G:$G,$F15)</f>
         <v>15</v>
       </c>
       <c r="F15">
@@ -11064,12 +11111,15 @@
         <v>10</v>
       </c>
       <c r="C16">
-        <v>121287644939.62</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A16,'Sheet1'!$C:$C,$B16,'Sheet1'!$G:$G,$F16)</f>
+        <v>121288000000</v>
       </c>
       <c r="D16">
-        <v>121287644939.62</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A16,'Sheet1'!$C:$C,$B16,'Sheet1'!$G:$G,$F16)</f>
+        <v>121288000000</v>
       </c>
       <c r="E16">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A16,'Sheet1'!$C:$C,$B16,'Sheet1'!$G:$G,$F16)</f>
         <v>173171</v>
       </c>
       <c r="F16">
@@ -11100,12 +11150,15 @@
         <v>10</v>
       </c>
       <c r="C17">
-        <v>210175711.440961</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A17,'Sheet1'!$C:$C,$B17,'Sheet1'!$G:$G,$F17)</f>
+        <v>210175711.428</v>
       </c>
       <c r="D17">
-        <v>112614669.916677</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A17,'Sheet1'!$C:$C,$B17,'Sheet1'!$G:$G,$F17)</f>
+        <v>112614669.918</v>
       </c>
       <c r="E17">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A17,'Sheet1'!$C:$C,$B17,'Sheet1'!$G:$G,$F17)</f>
         <v>11</v>
       </c>
       <c r="F17">
@@ -11136,12 +11189,15 @@
         <v>10</v>
       </c>
       <c r="C18">
-        <v>2859865269.6026502</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A18,'Sheet1'!$C:$C,$B18,'Sheet1'!$G:$G,$F18)</f>
+        <v>2859865269.5161</v>
       </c>
       <c r="D18">
-        <v>2193629057.13695</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A18,'Sheet1'!$C:$C,$B18,'Sheet1'!$G:$G,$F18)</f>
+        <v>2193629057.0861</v>
       </c>
       <c r="E18">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A18,'Sheet1'!$C:$C,$B18,'Sheet1'!$G:$G,$F18)</f>
         <v>612</v>
       </c>
       <c r="F18">
@@ -11172,12 +11228,15 @@
         <v>10</v>
       </c>
       <c r="C19">
-        <v>75479150.000190407</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A19,'Sheet1'!$C:$C,$B19,'Sheet1'!$G:$G,$F19)</f>
+        <v>75479150</v>
       </c>
       <c r="D19">
-        <v>75479150.000190407</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A19,'Sheet1'!$C:$C,$B19,'Sheet1'!$G:$G,$F19)</f>
+        <v>75479150</v>
       </c>
       <c r="E19">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A19,'Sheet1'!$C:$C,$B19,'Sheet1'!$G:$G,$F19)</f>
         <v>112</v>
       </c>
       <c r="F19">
@@ -11208,12 +11267,15 @@
         <v>10</v>
       </c>
       <c r="C20">
-        <v>56019841640.209999</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A20,'Sheet1'!$C:$C,$B20,'Sheet1'!$G:$G,$F20)</f>
+        <v>56019841640.34</v>
       </c>
       <c r="D20">
-        <v>54739890725.055099</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A20,'Sheet1'!$C:$C,$B20,'Sheet1'!$G:$G,$F20)</f>
+        <v>54739890726.34</v>
       </c>
       <c r="E20">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A20,'Sheet1'!$C:$C,$B20,'Sheet1'!$G:$G,$F20)</f>
         <v>67520</v>
       </c>
       <c r="F20">
@@ -11244,12 +11306,15 @@
         <v>11</v>
       </c>
       <c r="C21" s="1">
-        <v>3060082.6430000402</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A21,'Sheet1'!$C:$C,$B21,'Sheet1'!$G:$G,$F21)</f>
+        <v>3060082.643</v>
       </c>
       <c r="D21" s="1">
-        <v>1599407.4673806699</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A21,'Sheet1'!$C:$C,$B21,'Sheet1'!$G:$G,$F21)</f>
+        <v>1599407.467</v>
       </c>
       <c r="E21">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A21,'Sheet1'!$C:$C,$B21,'Sheet1'!$G:$G,$F21)</f>
         <v>3</v>
       </c>
       <c r="F21">
@@ -11280,12 +11345,15 @@
         <v>11</v>
       </c>
       <c r="C22" s="1">
-        <v>83586974.900705397</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A22,'Sheet1'!$C:$C,$B22,'Sheet1'!$G:$G,$F22)</f>
+        <v>83586974.9</v>
       </c>
       <c r="D22" s="1">
-        <v>47547710.997818798</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A22,'Sheet1'!$C:$C,$B22,'Sheet1'!$G:$G,$F22)</f>
+        <v>47547711</v>
       </c>
       <c r="E22">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A22,'Sheet1'!$C:$C,$B22,'Sheet1'!$G:$G,$F22)</f>
         <v>10</v>
       </c>
       <c r="F22">
@@ -11316,12 +11384,15 @@
         <v>11</v>
       </c>
       <c r="C23">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A23,'Sheet1'!$C:$C,$B23,'Sheet1'!$G:$G,$F23)</f>
         <v>276000</v>
       </c>
       <c r="D23">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A23,'Sheet1'!$C:$C,$B23,'Sheet1'!$G:$G,$F23)</f>
         <v>276000</v>
       </c>
       <c r="E23">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A23,'Sheet1'!$C:$C,$B23,'Sheet1'!$G:$G,$F23)</f>
         <v>2</v>
       </c>
       <c r="F23">
@@ -11352,12 +11423,15 @@
         <v>11</v>
       </c>
       <c r="C24">
-        <v>183525417.04899299</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A24,'Sheet1'!$C:$C,$B24,'Sheet1'!$G:$G,$F24)</f>
+        <v>183525417</v>
       </c>
       <c r="D24">
-        <v>107035050.91833501</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A24,'Sheet1'!$C:$C,$B24,'Sheet1'!$G:$G,$F24)</f>
+        <v>107035050.9</v>
       </c>
       <c r="E24">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A24,'Sheet1'!$C:$C,$B24,'Sheet1'!$G:$G,$F24)</f>
         <v>42</v>
       </c>
       <c r="F24">
@@ -11388,12 +11462,15 @@
         <v>11</v>
       </c>
       <c r="C25">
-        <v>20201080.800000001</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A25,'Sheet1'!$C:$C,$B25,'Sheet1'!$G:$G,$F25)</f>
+        <v>20201080.8</v>
       </c>
       <c r="D25">
-        <v>20201080.800000001</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A25,'Sheet1'!$C:$C,$B25,'Sheet1'!$G:$G,$F25)</f>
+        <v>20201080.8</v>
       </c>
       <c r="E25">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A25,'Sheet1'!$C:$C,$B25,'Sheet1'!$G:$G,$F25)</f>
         <v>23</v>
       </c>
       <c r="F25">
@@ -11424,12 +11501,15 @@
         <v>12</v>
       </c>
       <c r="C26" s="1">
-        <v>18301343.574820001</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A26,'Sheet1'!$C:$C,$B26,'Sheet1'!$G:$G,$F26)</f>
+        <v>18301343.57</v>
       </c>
       <c r="D26" s="1">
-        <v>16479715.6923308</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A26,'Sheet1'!$C:$C,$B26,'Sheet1'!$G:$G,$F26)</f>
+        <v>16479715.69</v>
       </c>
       <c r="E26">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A26,'Sheet1'!$C:$C,$B26,'Sheet1'!$G:$G,$F26)</f>
         <v>4</v>
       </c>
       <c r="F26">
@@ -11460,12 +11540,15 @@
         <v>12</v>
       </c>
       <c r="C27" s="1">
-        <v>210957528.07712299</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A27,'Sheet1'!$C:$C,$B27,'Sheet1'!$G:$G,$F27)</f>
+        <v>210957528.1</v>
       </c>
       <c r="D27" s="1">
-        <v>106631319.724132</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A27,'Sheet1'!$C:$C,$B27,'Sheet1'!$G:$G,$F27)</f>
+        <v>106631319.7</v>
       </c>
       <c r="E27">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A27,'Sheet1'!$C:$C,$B27,'Sheet1'!$G:$G,$F27)</f>
         <v>18</v>
       </c>
       <c r="F27">
@@ -11496,12 +11579,15 @@
         <v>12</v>
       </c>
       <c r="C28">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A28,'Sheet1'!$C:$C,$B28,'Sheet1'!$G:$G,$F28)</f>
         <v>110000</v>
       </c>
       <c r="D28">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A28,'Sheet1'!$C:$C,$B28,'Sheet1'!$G:$G,$F28)</f>
         <v>110000</v>
       </c>
       <c r="E28">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A28,'Sheet1'!$C:$C,$B28,'Sheet1'!$G:$G,$F28)</f>
         <v>1</v>
       </c>
       <c r="F28">
@@ -11532,12 +11618,15 @@
         <v>12</v>
       </c>
       <c r="C29">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A29,'Sheet1'!$C:$C,$B29,'Sheet1'!$G:$G,$F29)</f>
         <v>110000</v>
       </c>
       <c r="D29">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A29,'Sheet1'!$C:$C,$B29,'Sheet1'!$G:$G,$F29)</f>
         <v>110000</v>
       </c>
       <c r="E29">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A29,'Sheet1'!$C:$C,$B29,'Sheet1'!$G:$G,$F29)</f>
         <v>1</v>
       </c>
       <c r="F29">
@@ -11568,12 +11657,15 @@
         <v>12</v>
       </c>
       <c r="C30">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A30,'Sheet1'!$C:$C,$B30,'Sheet1'!$G:$G,$F30)</f>
         <v>212000</v>
       </c>
       <c r="D30">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A30,'Sheet1'!$C:$C,$B30,'Sheet1'!$G:$G,$F30)</f>
         <v>212000</v>
       </c>
       <c r="E30">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A30,'Sheet1'!$C:$C,$B30,'Sheet1'!$G:$G,$F30)</f>
         <v>1</v>
       </c>
       <c r="F30">
@@ -11604,12 +11696,15 @@
         <v>12</v>
       </c>
       <c r="C31">
-        <v>7558346.1603288203</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A31,'Sheet1'!$C:$C,$B31,'Sheet1'!$G:$G,$F31)</f>
+        <v>7558346.16</v>
       </c>
       <c r="D31">
-        <v>7558346.1603288203</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A31,'Sheet1'!$C:$C,$B31,'Sheet1'!$G:$G,$F31)</f>
+        <v>7558346.16</v>
       </c>
       <c r="E31">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A31,'Sheet1'!$C:$C,$B31,'Sheet1'!$G:$G,$F31)</f>
         <v>4</v>
       </c>
       <c r="F31">
@@ -11640,12 +11735,15 @@
         <v>12</v>
       </c>
       <c r="C32">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A32,'Sheet1'!$C:$C,$B32,'Sheet1'!$G:$G,$F32)</f>
         <v>560000</v>
       </c>
       <c r="D32">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A32,'Sheet1'!$C:$C,$B32,'Sheet1'!$G:$G,$F32)</f>
         <v>560000</v>
       </c>
       <c r="E32">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A32,'Sheet1'!$C:$C,$B32,'Sheet1'!$G:$G,$F32)</f>
         <v>2</v>
       </c>
       <c r="F32">
@@ -11676,12 +11774,15 @@
         <v>13</v>
       </c>
       <c r="C33" s="1">
-        <v>2372926089.2821898</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A33,'Sheet1'!$C:$C,$B33,'Sheet1'!$G:$G,$F33)</f>
+        <v>2372926089.373</v>
       </c>
       <c r="D33" s="1">
-        <v>1420410551.7284601</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A33,'Sheet1'!$C:$C,$B33,'Sheet1'!$G:$G,$F33)</f>
+        <v>1420410551.373</v>
       </c>
       <c r="E33">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A33,'Sheet1'!$C:$C,$B33,'Sheet1'!$G:$G,$F33)</f>
         <v>328</v>
       </c>
       <c r="F33">
@@ -11712,12 +11813,15 @@
         <v>13</v>
       </c>
       <c r="C34" s="1">
-        <v>761662142.94186294</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A34,'Sheet1'!$C:$C,$B34,'Sheet1'!$G:$G,$F34)</f>
+        <v>761662142.89</v>
       </c>
       <c r="D34" s="1">
-        <v>448941035.41101199</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A34,'Sheet1'!$C:$C,$B34,'Sheet1'!$G:$G,$F34)</f>
+        <v>448941035.39</v>
       </c>
       <c r="E34">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A34,'Sheet1'!$C:$C,$B34,'Sheet1'!$G:$G,$F34)</f>
         <v>119</v>
       </c>
       <c r="F34">
@@ -11748,12 +11852,15 @@
         <v>13</v>
       </c>
       <c r="C35">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A35,'Sheet1'!$C:$C,$B35,'Sheet1'!$G:$G,$F35)</f>
         <v>545000</v>
       </c>
       <c r="D35">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A35,'Sheet1'!$C:$C,$B35,'Sheet1'!$G:$G,$F35)</f>
         <v>545000</v>
       </c>
       <c r="E35">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A35,'Sheet1'!$C:$C,$B35,'Sheet1'!$G:$G,$F35)</f>
         <v>2</v>
       </c>
       <c r="F35">
@@ -11784,12 +11891,15 @@
         <v>13</v>
       </c>
       <c r="C36">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A36,'Sheet1'!$C:$C,$B36,'Sheet1'!$G:$G,$F36)</f>
         <v>2662700</v>
       </c>
       <c r="D36">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A36,'Sheet1'!$C:$C,$B36,'Sheet1'!$G:$G,$F36)</f>
         <v>2662700</v>
       </c>
       <c r="E36">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A36,'Sheet1'!$C:$C,$B36,'Sheet1'!$G:$G,$F36)</f>
         <v>4</v>
       </c>
       <c r="F36">
@@ -11820,12 +11930,15 @@
         <v>13</v>
       </c>
       <c r="C37">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A37,'Sheet1'!$C:$C,$B37,'Sheet1'!$G:$G,$F37)</f>
         <v>101000</v>
       </c>
       <c r="D37">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A37,'Sheet1'!$C:$C,$B37,'Sheet1'!$G:$G,$F37)</f>
         <v>101000</v>
       </c>
       <c r="E37">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A37,'Sheet1'!$C:$C,$B37,'Sheet1'!$G:$G,$F37)</f>
         <v>1</v>
       </c>
       <c r="F37">
@@ -11856,12 +11969,15 @@
         <v>13</v>
       </c>
       <c r="C38">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A38,'Sheet1'!$C:$C,$B38,'Sheet1'!$G:$G,$F38)</f>
         <v>22746034</v>
       </c>
       <c r="D38">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A38,'Sheet1'!$C:$C,$B38,'Sheet1'!$G:$G,$F38)</f>
         <v>22746034</v>
       </c>
       <c r="E38">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A38,'Sheet1'!$C:$C,$B38,'Sheet1'!$G:$G,$F38)</f>
         <v>32</v>
       </c>
       <c r="F38">
@@ -11892,12 +12008,15 @@
         <v>13</v>
       </c>
       <c r="C39">
-        <v>191741484.19769299</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A39,'Sheet1'!$C:$C,$B39,'Sheet1'!$G:$G,$F39)</f>
+        <v>191741484.23</v>
       </c>
       <c r="D39">
-        <v>103722848.999153</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A39,'Sheet1'!$C:$C,$B39,'Sheet1'!$G:$G,$F39)</f>
+        <v>103722849</v>
       </c>
       <c r="E39">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A39,'Sheet1'!$C:$C,$B39,'Sheet1'!$G:$G,$F39)</f>
         <v>23</v>
       </c>
       <c r="F39">
@@ -11928,12 +12047,15 @@
         <v>13</v>
       </c>
       <c r="C40">
-        <v>1205659420.18715</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A40,'Sheet1'!$C:$C,$B40,'Sheet1'!$G:$G,$F40)</f>
+        <v>1205659420.15</v>
       </c>
       <c r="D40">
-        <v>924487181.75075197</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A40,'Sheet1'!$C:$C,$B40,'Sheet1'!$G:$G,$F40)</f>
+        <v>924487181.77</v>
       </c>
       <c r="E40">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A40,'Sheet1'!$C:$C,$B40,'Sheet1'!$G:$G,$F40)</f>
         <v>318</v>
       </c>
       <c r="F40">
@@ -11964,12 +12086,15 @@
         <v>13</v>
       </c>
       <c r="C41">
-        <v>107224705.21595199</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A41,'Sheet1'!$C:$C,$B41,'Sheet1'!$G:$G,$F41)</f>
+        <v>107224705.2</v>
       </c>
       <c r="D41">
-        <v>106417749.21595199</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A41,'Sheet1'!$C:$C,$B41,'Sheet1'!$G:$G,$F41)</f>
+        <v>106417749.2</v>
       </c>
       <c r="E41">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A41,'Sheet1'!$C:$C,$B41,'Sheet1'!$G:$G,$F41)</f>
         <v>86</v>
       </c>
       <c r="F41">
@@ -12000,12 +12125,15 @@
         <v>14</v>
       </c>
       <c r="C42" s="1">
-        <v>2365811502.90905</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A42,'Sheet1'!$C:$C,$B42,'Sheet1'!$G:$G,$F42)</f>
+        <v>2365811503</v>
       </c>
       <c r="D42" s="1">
-        <v>1413295965.35532</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A42,'Sheet1'!$C:$C,$B42,'Sheet1'!$G:$G,$F42)</f>
+        <v>1413295965</v>
       </c>
       <c r="E42">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A42,'Sheet1'!$C:$C,$B42,'Sheet1'!$G:$G,$F42)</f>
         <v>326</v>
       </c>
       <c r="F42">
@@ -12036,12 +12164,15 @@
         <v>14</v>
       </c>
       <c r="C43" s="1">
-        <v>738973417.34851599</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A43,'Sheet1'!$C:$C,$B43,'Sheet1'!$G:$G,$F43)</f>
+        <v>738973417.3</v>
       </c>
       <c r="D43" s="1">
-        <v>426252309.81766498</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A43,'Sheet1'!$C:$C,$B43,'Sheet1'!$G:$G,$F43)</f>
+        <v>426252309.8</v>
       </c>
       <c r="E43">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A43,'Sheet1'!$C:$C,$B43,'Sheet1'!$G:$G,$F43)</f>
         <v>106</v>
       </c>
       <c r="F43">
@@ -12072,12 +12203,15 @@
         <v>14</v>
       </c>
       <c r="C44">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A44,'Sheet1'!$C:$C,$B44,'Sheet1'!$G:$G,$F44)</f>
         <v>345000</v>
       </c>
       <c r="D44">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A44,'Sheet1'!$C:$C,$B44,'Sheet1'!$G:$G,$F44)</f>
         <v>345000</v>
       </c>
       <c r="E44">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A44,'Sheet1'!$C:$C,$B44,'Sheet1'!$G:$G,$F44)</f>
         <v>1</v>
       </c>
       <c r="F44">
@@ -12108,12 +12242,15 @@
         <v>14</v>
       </c>
       <c r="C45">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A45,'Sheet1'!$C:$C,$B45,'Sheet1'!$G:$G,$F45)</f>
         <v>2462700</v>
       </c>
       <c r="D45">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A45,'Sheet1'!$C:$C,$B45,'Sheet1'!$G:$G,$F45)</f>
         <v>2462700</v>
       </c>
       <c r="E45">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A45,'Sheet1'!$C:$C,$B45,'Sheet1'!$G:$G,$F45)</f>
         <v>3</v>
       </c>
       <c r="F45">
@@ -12144,12 +12281,15 @@
         <v>14</v>
       </c>
       <c r="C46">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A46,'Sheet1'!$C:$C,$B46,'Sheet1'!$G:$G,$F46)</f>
         <v>101000</v>
       </c>
       <c r="D46">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A46,'Sheet1'!$C:$C,$B46,'Sheet1'!$G:$G,$F46)</f>
         <v>101000</v>
       </c>
       <c r="E46">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A46,'Sheet1'!$C:$C,$B46,'Sheet1'!$G:$G,$F46)</f>
         <v>1</v>
       </c>
       <c r="F46">
@@ -12180,12 +12320,15 @@
         <v>14</v>
       </c>
       <c r="C47">
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A47,'Sheet1'!$C:$C,$B47,'Sheet1'!$G:$G,$F47)</f>
         <v>22746034</v>
       </c>
       <c r="D47">
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A47,'Sheet1'!$C:$C,$B47,'Sheet1'!$G:$G,$F47)</f>
         <v>22746034</v>
       </c>
       <c r="E47">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A47,'Sheet1'!$C:$C,$B47,'Sheet1'!$G:$G,$F47)</f>
         <v>32</v>
       </c>
       <c r="F47">
@@ -12216,12 +12359,15 @@
         <v>14</v>
       </c>
       <c r="C48">
-        <v>175292598.767708</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A48,'Sheet1'!$C:$C,$B48,'Sheet1'!$G:$G,$F48)</f>
+        <v>175292598.8</v>
       </c>
       <c r="D48">
-        <v>87273963.569168001</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A48,'Sheet1'!$C:$C,$B48,'Sheet1'!$G:$G,$F48)</f>
+        <v>87273963.57</v>
       </c>
       <c r="E48">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A48,'Sheet1'!$C:$C,$B48,'Sheet1'!$G:$G,$F48)</f>
         <v>20</v>
       </c>
       <c r="F48">
@@ -12252,12 +12398,15 @@
         <v>14</v>
       </c>
       <c r="C49">
-        <v>906507554.61050797</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A49,'Sheet1'!$C:$C,$B49,'Sheet1'!$G:$G,$F49)</f>
+        <v>906507554.6</v>
       </c>
       <c r="D49">
-        <v>666539312.39975405</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A49,'Sheet1'!$C:$C,$B49,'Sheet1'!$G:$G,$F49)</f>
+        <v>666539312.4</v>
       </c>
       <c r="E49">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A49,'Sheet1'!$C:$C,$B49,'Sheet1'!$G:$G,$F49)</f>
         <v>227</v>
       </c>
       <c r="F49">
@@ -12288,12 +12437,15 @@
         <v>14</v>
       </c>
       <c r="C50">
-        <v>101774358.815952</v>
+        <f>SUMIFS('Sheet1'!$D:$D,'Sheet1'!$B:$B,$A50,'Sheet1'!$C:$C,$B50,'Sheet1'!$G:$G,$F50)</f>
+        <v>101774358.8</v>
       </c>
       <c r="D50">
-        <v>100967402.815952</v>
+        <f>SUMIFS('Sheet1'!$E:$E,'Sheet1'!$B:$B,$A50,'Sheet1'!$C:$C,$B50,'Sheet1'!$G:$G,$F50)</f>
+        <v>100967402.8</v>
       </c>
       <c r="E50">
+        <f>SUMIFS('Sheet1'!$F:$F,'Sheet1'!$B:$B,$A50,'Sheet1'!$C:$C,$B50,'Sheet1'!$G:$G,$F50)</f>
         <v>76</v>
       </c>
       <c r="F50">
@@ -12536,11 +12688,11 @@
         <v>0</v>
       </c>
       <c r="H2" s="7">
-        <f>D2*1.35</f>
+        <f>D2*Settings!$B$3</f>
         <v>18149996.794500001</v>
       </c>
       <c r="I2" s="1">
-        <f>E2*1.35</f>
+        <f>E2*Settings!$B$3</f>
         <v>14681118.037500001</v>
       </c>
       <c r="J2" s="7">
@@ -30915,6 +31067,778 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="82" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BSCR workbook settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FX rate: source currency to USD</t>
+        </is>
+      </c>
+      <c r="B3" s="7">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Source currency</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Output currency</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Output unit</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>USD millions</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Formula note</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Change Settings!B3 to update source/output conversions and schedule-input tabs.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.3" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D14"/>
+  <cols>
+    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="58" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CATASTROPHE RISK RETURN: EP CURVE TOTAL INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Only source-supported reference exposure is shown; EP-curve values remain blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Required input</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Gross</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>50-year TVaR</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>100-year TVaR</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>250-year TVaR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>500-year TVaR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1000-year TVaR</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Annual average aggregate loss</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Standard deviation of annual aggregate loss</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Property catastrophe premium</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>All other catastrophe premium</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Reference: HIC all-region exposure limit</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <v>164353.167868337</v>
+      </c>
+      <c r="C14" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <v>164353.167868337</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Exposure reference only; not an EP-curve input</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.3" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D14"/>
+  <cols>
+    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="58" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CATASTROPHE RISK RETURN: EP CURVE INSURANCE INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Insurance EP-curve and premium values are not produced by the BSCR exposure output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Required input</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Gross</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>50-year TVaR</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>100-year TVaR</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>250-year TVaR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>500-year TVaR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1000-year TVaR</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Annual average aggregate loss</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Standard deviation of annual aggregate loss</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Property catastrophe premium</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>All other catastrophe premium</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model or premium source</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Reference: HIC all-region exposure limit</t>
+        </is>
+      </c>
+      <c r="B14" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <v>164353.167868337</v>
+      </c>
+      <c r="C14" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <v>164353.167868337</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Exposure reference only; not an EP-curve input</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.3" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D12"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="62" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CATASTROPHE RISK RETURN: REGIONS-PERILS INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exposure limits sourced from HIC output; amounts are USD millions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Gross</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Source / status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Atlantic Basin Hurricane</t>
+        </is>
+      </c>
+      <c r="B4" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_nahu")</f>
+        <v>30.8434959</v>
+      </c>
+      <c r="C4" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_nahu")</f>
+        <v>30.8434959</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>HIC output region total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>North American Earthquake</t>
+        </is>
+      </c>
+      <c r="B5" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_na_eq")</f>
+        <v>0.2862</v>
+      </c>
+      <c r="C5" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_na_eq")</f>
+        <v>0.2862</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>HIC output region total</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>European Windstorm</t>
+        </is>
+      </c>
+      <c r="B6" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_eu")</f>
+        <v>163747.905595587</v>
+      </c>
+      <c r="C6" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_eu")</f>
+        <v>163747.905595587</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>HIC output region total</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Japanese Earthquake</t>
+        </is>
+      </c>
+      <c r="B7" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <v>0.3726</v>
+      </c>
+      <c r="C7" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <v>0.3726</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>HIC output region total</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Japanese Typhoon</t>
+        </is>
+      </c>
+      <c r="B8" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <v>0.3726</v>
+      </c>
+      <c r="C8" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_jp")</f>
+        <v>0.3726</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Uses Japanese earthquake region; separate typhoon split unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Premium inputs</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Not supplied by the BSCR exposure output</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>EP curve loss inputs</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Requires catastrophe model output</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.3" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H8"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CATASTROPHE RISK RETURN: DATA ANALYSIS INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exposure summary; modelability classifications are not available in the BSCR output</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>US count</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>US gross (US$M)</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>US net (US$M)</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>All-other count</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>All-other gross (US$M)</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>All-other net (US$M)</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>All contracts - geographic split only</t>
+        </is>
+      </c>
+      <c r="B4" s="7">
+        <f>SUMIFS('output'!$E:$E,'output'!$A:$A,"HIC",'output'!$B:$B,"is_us_all")</f>
+        <v>33</v>
+      </c>
+      <c r="C4" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"is_us_all")</f>
+        <v>30.8434959</v>
+      </c>
+      <c r="D4" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"is_us_all")</f>
+        <v>30.8434959</v>
+      </c>
+      <c r="E4" s="7">
+        <f>SUMIFS('output'!$E:$E,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")-B4</f>
+        <v>173654</v>
+      </c>
+      <c r="F4" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")-C4</f>
+        <v>164322.324372437</v>
+      </c>
+      <c r="G4" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")-D4</f>
+        <v>164322.324372437</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Not a modelled/not-modelled classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Modelled</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Requires approved modelability classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Not modelled</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Requires approved modelability classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Control: HIC total output</t>
+        </is>
+      </c>
+      <c r="B8" s="7">
+        <f>SUMIFS('output'!$E:$E,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <v>173687</v>
+      </c>
+      <c r="C8" s="7">
+        <f>SUMIFS('output'!$I:$I,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <v>164353.167868337</v>
+      </c>
+      <c r="D8" s="7">
+        <f>SUMIFS('output'!$J:$J,'output'!$A:$A,"HIC",'output'!$B:$B,"ALL")</f>
+        <v>164353.167868337</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Control total</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.3" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{b0e772fd-230e-46a1-9b91-16e31ba7e038}" enabled="1" method="Privileged" siteId="{dfbcc178-bccf-4595-8f8e-3a3175df90b7}" contentBits="0" removed="0"/>

</xml_diff>